<commit_message>
moved the exiftool metadata extraction to iramat-functions
</commit_message>
<xml_diff>
--- a/iiif/metadata.xlsx
+++ b/iiif/metadata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TH282424\Rprojects\iramat-dev\iiif\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F499B8D1-665B-4D21-9998-3041F3A7BDC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{674B0D96-F42D-4691-B4D1-5A201D95E957}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28692" yWindow="-108" windowWidth="25416" windowHeight="15252" xr2:uid="{39E1CB0A-AB15-4586-9A56-B91CD41D8965}"/>
   </bookViews>
@@ -140,14 +140,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -188,12 +181,12 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -202,7 +195,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -586,7 +579,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" hidden="1">
       <c r="A5" s="4" t="s">
         <v>11</v>
       </c>
@@ -614,7 +607,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:4" hidden="1">
       <c r="A7" s="4" t="s">
         <v>17</v>
       </c>

</xml_diff>